<commit_message>
Added Jupyter notebook along with the pdf output
</commit_message>
<xml_diff>
--- a/output/AutoEIT_Transcriptions_Complete.xlsx
+++ b/output/AutoEIT_Transcriptions_Complete.xlsx
@@ -6342,7 +6342,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Me gustaría los precios de las caras para nada.</t>
+          <t>a nosotros que las vistas</t>
         </is>
       </c>
     </row>
@@ -6357,7 +6357,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Ellas solo beben cerveza y no comen nada.</t>
+          <t>ellas solo beben cerveza</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Me gustaría que el precio de las casas bajara.</t>
+          <t>Me gustaría los precios de las caras para nada.</t>
         </is>
       </c>
     </row>
@@ -6402,7 +6402,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Ella ha terminado de pintar su apartamento.</t>
+          <t>Ella ha terminado los apartamentos.</t>
         </is>
       </c>
     </row>
@@ -6447,7 +6447,7 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Una amiga bien cuidar a los niños a mi vecino.</t>
+          <t>Una amiga bien cuidar los niños a mi vecino.</t>
         </is>
       </c>
     </row>
@@ -11480,7 +11480,7 @@
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>Quiero cortar el pelo.</t>
+          <t>qui из-ste libra</t>
         </is>
       </c>
     </row>
@@ -11495,7 +11495,7 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>se han de poner a la mesa</t>
+          <t>El libro está en la mesa.</t>
         </is>
       </c>
       <c r="F3" s="16" t="inlineStr">
@@ -11515,7 +11515,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Ellas Metro los Langi segreseros</t>
+          <t>El carro lo tiene a pelo.</t>
         </is>
       </c>
       <c r="F4" s="16" t="inlineStr">
@@ -11535,7 +11535,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>El chico è spagnolo</t>
+          <t>Él se duche cada mañana.</t>
         </is>
       </c>
       <c r="F5" s="18" t="inlineStr">
@@ -11555,7 +11555,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>En Bub Janet si no hundred, que esta en la mesa.....el libro....</t>
+          <t>Me siento no voy a superpower.</t>
         </is>
       </c>
     </row>
@@ -11570,7 +11570,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Saben que soy una respeto, así que 걸 conmigo.</t>
+          <t>[no response detected]</t>
         </is>
       </c>
     </row>
@@ -11585,7 +11585,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Ya sé lo de la situación aquí.</t>
+          <t>Los calla santo.</t>
         </is>
       </c>
     </row>
@@ -11600,7 +11600,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Así que volviendo aquí.</t>
+          <t>Vuelvo a punto de entender.</t>
         </is>
       </c>
     </row>
@@ -11630,7 +11630,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Me gusta las películas peca bien.</t>
+          <t>Me gustan las películas pegar bien.</t>
         </is>
       </c>
     </row>
@@ -11645,7 +11645,7 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Son cosas que no mecolates a mí.</t>
+          <t>El chico es mono español.</t>
         </is>
       </c>
     </row>
@@ -11660,7 +11660,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Después llegar dormir</t>
+          <t>Después de llegar dormía.</t>
         </is>
       </c>
     </row>
@@ -11675,7 +11675,7 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>está a mi animales</t>
+          <t>Quiero la casa esta a mi animales.</t>
         </is>
       </c>
     </row>
@@ -11690,7 +11690,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>A nosotras fascinabas a los nosotros</t>
+          <t>A nosotros fascinabas a los nosotros.</t>
         </is>
       </c>
     </row>
@@ -11705,7 +11705,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Ellas elps inconversi nos del do pi casam</t>
+          <t>Ambassador Myrtle Perkins es el conversino de donde estamos.</t>
         </is>
       </c>
     </row>
@@ -11720,7 +11720,7 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Me gustaría que los brazos me estaban cruzando a la derecha.</t>
+          <t>Me gustaría que los huesos bestas cruzaran a la derecha.</t>
         </is>
       </c>
     </row>
@@ -11735,7 +11735,7 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>[no response detected]</t>
+          <t>Una chica picarettes pisástico.</t>
         </is>
       </c>
     </row>
@@ -11750,7 +11750,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>He terminado despacxy la cr Testament</t>
+          <t>He terminado el fragmento.</t>
         </is>
       </c>
     </row>
@@ -11765,7 +11765,7 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Me gustaria hacer pingatasasonic visitas a pandemic</t>
+          <t>Me gustaría hacer pintadas por esta, muy pronto.</t>
         </is>
       </c>
     </row>
@@ -11780,7 +11780,7 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>El nino sirio es tan muy triste.</t>
+          <t>El niño.. El niño Serio Cato es muy triste.</t>
         </is>
       </c>
     </row>
@@ -11795,7 +11795,7 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Una amiga picabon en la saritana.</t>
+          <t>Una amiga picandro en mi vecino...</t>
         </is>
       </c>
     </row>
@@ -11810,7 +11810,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>El cato tiene cin Chef de r, te hace muy frúcar.</t>
+          <t>El gato tenga nemi, i la perla.</t>
         </is>
       </c>
     </row>
@@ -11825,7 +11825,7 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Te ha ware mi Hol equal se heck skim.</t>
+          <t>[no response detected]</t>
         </is>
       </c>
     </row>
@@ -11840,7 +11840,7 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>La cantina layas recycling esa persona a mi casa Ah</t>
+          <t>[no response detected]</t>
         </is>
       </c>
     </row>
@@ -11855,7 +11855,7 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>ahora le voy a la cena</t>
+          <t>Después de llegar a mi casa, voy a la cena.</t>
         </is>
       </c>
     </row>
@@ -11870,7 +11870,7 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>policía era famoso</t>
+          <t>El pueblo se que ella calla.</t>
         </is>
       </c>
     </row>
@@ -11885,7 +11885,7 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Ya sé qué cont hemen con la Pis.</t>
+          <t>Una estaban viendo del software cuando decían con la cara así .</t>
         </is>
       </c>
     </row>
@@ -11900,7 +11900,7 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Entonces la tarea esta no difícil, pero debe ser.</t>
+          <t>El tarea esta no difícil pero...</t>
         </is>
       </c>
     </row>
@@ -11915,7 +11915,7 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Las traen un seaswell tu se samg six xen.</t>
+          <t>están en la mesa</t>
         </is>
       </c>
     </row>
@@ -11930,7 +11930,7 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>hay muchos ejemplos</t>
+          <t>Hay muchos ejemplos, pero...</t>
         </is>
       </c>
     </row>
@@ -16828,7 +16828,7 @@
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>[no response detected]</t>
+          <t>¿Qué dice usted que va a ser hoy?</t>
         </is>
       </c>
       <c r="G2" s="18" t="inlineStr">
@@ -16893,7 +16893,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>¿Qué dice usted es que va a ser hoy?</t>
+          <t>¿Qué dice usted que va a ser hoy?</t>
         </is>
       </c>
     </row>

</xml_diff>